<commit_message>
Update ignore lists and correct spelling errors in course documents
- Added new terms to SV_IGNORE and EN_IGNORE lists in checks_common.py.
- Updated various Excel files related to grading scales, examination forms, and Bloom's taxonomy across IIT, IHV, IKS, and ISLL directories.
- Corrected spelling errors in the Stavfel och språkbruk.md and corresponding Excel files, including adjustments to download links and counts.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1039,12 +1039,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>GMT3JT</t>
+          <t>AEG225</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1054,24 +1054,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>`eu-förordningen` (sv)</t>
+          <t>`produktionskattelättnader` (sv)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JT</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>MT1060</t>
+          <t>AEG22R</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1081,46 +1081,46 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>`vridspänningar` (sv)</t>
+          <t>`mättteknik` (sv)</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>MT2006</t>
+          <t>AEG2AL</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>`höckerlind` (sv)</t>
+          <t>`andrelate` (en)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT2006</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>AEG225</t>
+          <t>AEG2AQ</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1130,24 +1130,24 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>`produktionskattelättnader` (sv)</t>
+          <t>`adress` (en)</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AQ</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>AEG225</t>
+          <t>AEG2AW</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1157,24 +1157,24 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>`softlån` (sv)</t>
+          <t>`wich` (en)</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG225</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AW</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>AEG22R</t>
+          <t>AEG2AY</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1189,19 +1189,19 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>`mättteknik` (sv)</t>
+          <t>`inlämninguppgifter` (sv)</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG22R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AY</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>AEG2AL</t>
+          <t>AEG2C5</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1216,19 +1216,19 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>`andrelate` (en)</t>
+          <t>`laboatory` (en)</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AL</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2C5</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>AEG2AQ</t>
+          <t>EG3007</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1243,19 +1243,19 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>`adress` (en)</t>
+          <t>`absorbers` (en)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>AEG2AW</t>
+          <t>EG3014</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1270,19 +1270,19 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>`wich` (en)</t>
+          <t>`appropiate` (en)</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AW</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>AEG2AY</t>
+          <t>EG3014</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1292,24 +1292,24 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>`inlämninguppgifter` (sv)</t>
+          <t>`crediits` (en)</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AY</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>AEG2C5</t>
+          <t>EG3015</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1324,19 +1324,19 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>`laboatory` (en)</t>
+          <t>`horizontoscope` (en)</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2C5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>EG3007</t>
+          <t>EG3017</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1346,24 +1346,24 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>`absorbers` (en)</t>
+          <t>`genomförds` (sv)</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3007</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>EG3014</t>
+          <t>EG3018</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1373,24 +1373,24 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>`appropiate` (en)</t>
+          <t>`genomförds` (sv)</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>EG3014</t>
+          <t>EG4001</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1405,19 +1405,19 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>`crediits` (en)</t>
+          <t>`continuewith` (en)</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3014</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG4001</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>EG3015</t>
+          <t>EG4001</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1432,19 +1432,19 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>`horizontoscope` (en)</t>
+          <t>`fulltime` (en)</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3015</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG4001</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>EG3017</t>
+          <t>GEG26J</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1454,24 +1454,24 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>`genomförds` (sv)</t>
+          <t>`tutoria` (en)</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3017</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>EG3018</t>
+          <t>GEG2ZQ</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1486,19 +1486,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>`genomförds` (sv)</t>
+          <t>`inlämninguppgifter` (sv)</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG3018</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZQ</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>EG4001</t>
+          <t>GEG2ZR</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1508,83 +1508,83 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>`continuewith` (en)</t>
+          <t>`inlämingsuppgifter` (sv)</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG4001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZR</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>EG4001</t>
+          <t>GSQ25J</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Dubblerat ord</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>`fulltime` (en)</t>
+          <t>`hp` — …ch skriftliga inlämningsuppgifter i kvantitativa metoder, 4 hp hp  ## Arbetsformer  Föreläsningar, seminarier och övningar.…</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG4001</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25J</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>GEG26J</t>
+          <t>GSQ25K</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Felstavning (en)</t>
+          <t>Felstavning</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>`tutoria` (en)</t>
+          <t>`skalniåver` (sv)</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG26J</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>GEG2ZQ</t>
+          <t>GSQ33N</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1594,287 +1594,98 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>`inlämninguppgifter` (sv)</t>
+          <t>`skalniåver` (sv)</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ33N</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>GEG2ZQ</t>
+          <t>GMI23G</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>`solcellsanläggingar` (sv)</t>
+          <t>`eulides` (en)</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>GEG2ZQ</t>
+          <t>GMI2C8</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>`solstrålsberäkningar` (sv)</t>
+          <t>`mathodology` (en)</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2C8</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>GEG2ZR</t>
+          <t>GMI2J3</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>`inlämingsuppgifter` (sv)</t>
+          <t>`discusess` (en)</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZR</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>GSQ25J</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>SQQ</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Dubblerat ord</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>`hp` — …ch skriftliga inlämningsuppgifter i kvantitativa metoder, 4 hp hp  ## Arbetsformer  Föreläsningar, seminarier och övningar.…</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25J</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>GSQ25K</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>SQQ</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>`gis-övningar` (sv)</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>GSQ25K</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>SQQ</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>`skalniåver` (sv)</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>GSQ33N</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>SQQ</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>`skalniåver` (sv)</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ33N</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>GMI23G</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>`eulides` (en)</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>GMI2C8</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>`mathodology` (en)</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2C8</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>GMI2J3</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>`discusess` (en)</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2J3</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E53"/>
+  <autoFilter ref="A1:E46"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -1966,20 +1777,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId88"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId89"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A48" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A50" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A51" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A53" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId104"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update course information and correct errors in various MOC documents
- Adjusted course counts and details in IKS MOC and ISLL MOC documents.
- Updated course lists in "Entreprenörskap och innovationsteknik", "Ljud- och musikproduktion", "Franska", and "Kinesiska" MOC files.
- Corrected spelling errors and inconsistencies in the "Stavfel och språkbruk" analysis documents.
- Updated binary files for analysis spreadsheets in both IKS and ISLL sections.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -472,93 +472,35 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GMA2EY</t>
+          <t>GSQ23K</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MAA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Felstavning</t>
+          <t>Felstavning (en)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>`indicies` → indices (en)</t>
+          <t>`credtis` (en)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMA2EY</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>GEG2ZQ</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>MÖY</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>`solcellsanläggingar` → solcellsanläggningar</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG2ZQ</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>GMI2C8</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>`mathodology` (en)</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI2C8</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E4"/>
+  <autoFilter ref="A1:E2"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId6"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update analysis documents and correct spelling errors in course plans
- Modified the "Stavfel och språkbruk" Excel files in both IKS and ISLL directories to reflect updated data.
- Updated the "Terminologi" Excel files in both IKS and ISLL directories with new terminology.
- Revised the "Övrigt" Excel files in both IKS and ISLL directories for consistency.
- Enhanced the "Betygsrapportering", "Betygsskalor", "Bloom-taxonomi", "Examinationsformer", and "Frasningskonsistens" Excel files in the ISLL directory to include additional analysis.
- Updated the "Förkunskapskrav" Markdown and Excel files in the ISLL directory to improve clarity and relevance.
- Revised the "Innehåll" Excel file in the ISLL directory for better content organization.
- Corrected spelling errors and improved formatting in the "Stavfel och språkbruk" Markdown file in the ISLL directory.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +30,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -55,11 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -462,7 +469,39 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>GSQ23K</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Felstavning (en)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>`credtis` (en)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:E2"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update various analysis files in the ISLL project
- Modified the content of the following Excel files:
  - Färkunskapskrav.xlsx
  - Innehåll.xlsx
  - Introfras.xlsx
  - Omfång på lärandemål.xlsx
  - Samstämmighet svenska och engelska.xlsx
  - Stavfel och språkbruk.xlsx
  - Terminologi.xlsx
  - Övrigt.xlsx

- Updated the Markdown file Stavfel och språkbruk.md to reflect changes in the analysis data, including a reduction in the number of findings from 122 to 5.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$2</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,10 +28,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <color rgb="000563C1"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -61,12 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -469,39 +462,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>GSQ23K</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>SQQ</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>`credtis` (en)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E2"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update analysis files for Dalarna University courses
- Modified "Stavfel och språkbruk" analysis in both ISLL and IKS folders, updating the Excel files and the corresponding markdown documentation to reflect the latest findings and corrections.
- Updated terminology and additional analysis files across various subjects, ensuring all relevant data is current and accurately represented.
- Adjusted links and content in markdown files to match the new data in the Excel sheets, enhancing clarity and accessibility for users.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +30,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -55,11 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -462,7 +469,39 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>GSQ23K</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Felstavning (en)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>`credtis` (en)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:E2"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update course plans and analysis documents for IKS and ISLL
- Modified course plan for Företagsekonomi (GFÖ3FJ) by removing 'vilande' tag.
- Added a new course (GLP2MU) to the Ljud- och musikproduktion MOC, increasing total courses to 14.
- Updated Medieproduktion MOC by adding a new course (GMN3JF) and adjusting the count of active and dormant courses.
- Enhanced Statsvetenskap MOC with a new course (ASK289) and updated dormant course count.
- Updated various analysis Excel files in ISLL, indicating changes in content.
- Revised Stavfel och språkbruk document to reflect an increase in identified issues from 5 to 122.
- Adjusted Kinesiska MOC by adding a new course (AKI2BN) and updating the count of dormant courses.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +30,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -55,11 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -462,7 +469,39 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>GSQ23K</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Felstavning (en)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>`credtis` (en)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:E2"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update analysis files across multiple departments with revised content and corrections
- Updated Betygsrapportering, Betygsskalor, Bloom-taxonomi, Examinationsformer, Frasningskonsistens, Färkunskapskrav, Introfras, Nedlagda kursreferenser, Omfång på lärandemål, Samstämmighet svenska och engelska, Stavfel och språkbruk, and Övrigt files in 01 IIT, 02 IHV, 03 IKS, and 04 ISLL directories.
- Adjusted download links and row counts in Stavfel och språkbruk markdown files.
- Corrected spelling errors and inconsistencies in course plans.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$8</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,10 +28,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <color rgb="000563C1"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -61,12 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -469,213 +462,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>DITMG</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>`mjukvarutestningsområdena` (sv)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DITMG</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>DITMG</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>`mjukvarutestningsområdet` (sv)</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DITMG</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>DSVPG</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>`pär` (sv)</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DSVPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>TTBRB</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>`förutbildningen` (sv)</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TTBRB</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>TTBRB</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>`römsing` (sv)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TTBRB</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>TTEKB</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>`förutbildningen` (sv)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TTEKB</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>TTEKB</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>`römsing` (sv)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TTEKB</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E8"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId14"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: update analysis Excel files and remove obsolete record
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -472,12 +472,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>FDA222R</t>
+          <t>FMI2222</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ANALYTIC</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -487,24 +487,24 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>`contextualise` (en)</t>
+          <t>`experiental` (en)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222R</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2222</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>FDA222S</t>
+          <t>FMI2224</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ANALYTIC</t>
+          <t>MIKRODAT</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -514,225 +514,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>`backpropagation` (en)</t>
+          <t>`seperability` (en)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222S</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>FDA222S</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>ANALYTIC</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>`feedforward` (en)</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222S</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>FDA222S</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>ANALYTIC</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>`rnns` (en)</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FDA222S</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>FEB222L</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>ENERGIBM</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>`prosumers` (en)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222L</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>FEB222Q</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ENERGIBM</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>`contextualise` (en)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222Q</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>FEB222Q</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>ENERGIBM</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>`transdisciplinary` (en)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FEB222Q</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>FMI2222</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>MIKRODAT</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>`experiental` (en)</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2222</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>FMI2224</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>MIKRODAT</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>`seperability` (en)</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2224</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E10"/>
+  <autoFilter ref="A1:E3"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId18"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add new Excel file for Programkurser analysis in Dalarna University vault
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$E$8</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,10 +28,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <color rgb="000563C1"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -61,12 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -469,213 +462,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>DITMG</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>`mjukvarutestningsområdena` (sv)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DITMG</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>DITMG</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>`mjukvarutestningsområdet` (sv)</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DITMG</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>DSVPG</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>`pär` (sv)</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DSVPG</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>TTBRB</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>`förutbildningen` (sv)</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TTBRB</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>TTBRB</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>`römsing` (sv)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TTBRB</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>TTEKB</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>`förutbildningen` (sv)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TTEKB</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>TTEKB</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Utbildningsplaner</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Felstavning</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>`römsing` (sv)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TTEKB</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E8"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId14"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update course plans and analysis notes for ISLL programs
- Updated course descriptions and main areas for various languages including Arabic, English, French, Italian, Japanese, Chinese, Portuguese, Russian, Spanish, Swedish, and German.
- Added quality notes regarding unlinked courses and discrepancies in course names for multiple educational plans (e.g., HSVAA, HTESA, LG79A, LGGYA, LL46A, LLF3A, LLL3A, LLL6A, LLP6A, LU79A, LUGYA, LYSLA).
- Adjusted the formatting and content of the ISLL markdown files to enhance clarity and accuracy.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$G$3</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,10 +28,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <color rgb="000563C1"/>
-      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -61,12 +55,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -432,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -481,80 +474,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>FMI2222</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>MIKRODAT</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>2019-10-03</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>`experiental` (en)</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2222</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>FMI2224</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>MIKRODAT</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2019-10-29</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Felstavning (en)</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>`seperability` (en)</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FMI2224</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G3"/>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update course plans and assessment methods for various courses in IIT and MTA
- Modified course descriptions and learning outcomes for GIE3JW, GMT3JQ, GMT3JR, GMT3JT, GMT3JU, GMT3JV, and GMT3JY to enhance clarity and consistency.
- Updated assessment methods to include individual assessments for written and oral exams across multiple courses.
- Corrected spelling and grammatical errors in course content and learning outcomes.
- Added quality notes for course plans highlighting areas for improvement.
- Adjusted course names for consistency in capitalization and terminology.
- Updated scrape hashes for all modified course plans.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$G$5</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,6 +30,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -55,11 +61,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -474,7 +481,150 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>GIE3JS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>IEA</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Felstavning (en)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>`understandingwithin` (en)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE3JS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>GMT3JR</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Felstavning (en)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>`mechanicsthe` (en)</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JR</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>GMT3JR</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2026-03-30</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Felstavning (en)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>`vapours` (en)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JR</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>GMT3JV</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Felstavning (en)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>`assessmen` (en)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMT3JV</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:G5"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId8"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update various analysis and course plan files across multiple programs
- Modified Excel files related to Bloom's taxonomy, examination forms, and consistency analysis for courses in the IHV, IKS, and ISLL programs.
- Updated markdown files for course plans, including changes in course names, descriptions, and course codes.
- Adjusted the number of courses listed in the markdown files for the Pedagogiskt arbete and Rättsvetenskap subjects.
- Corrected download links and descriptions in the Vilande kursplaner markdown file.
- Added program responsible name in the LGGYA program plan.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Stavfel och språkbruk.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Stavfel och språkbruk" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$G$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Stavfel och språkbruk'!$A$1:$G$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -613,8 +613,41 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>GEG3K9</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Felstavning (en)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>`thebasic` (en)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3K9</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G5"/>
+  <autoFilter ref="A1:G6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
@@ -624,6 +657,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId7"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>